<commit_message>
Listo para pruebas piloto
</commit_message>
<xml_diff>
--- a/evaluation/cuestionarios_participante.xlsx
+++ b/evaluation/cuestionarios_participante.xlsx
@@ -737,10 +737,10 @@
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>No importa la redacción: puedes escribir oraciones o una lista de ideas. Si de una página no recuerdas nada, escribe «No recuerdo».</t>
+          <t>Las páginas están en el orden en que las leíste: la página web 1 es la primera. No importa la redacción: oraciones o una lista de ideas. Si de una página no recuerdas nada, escribe «No recuerdo».</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -764,7 +764,7 @@
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Página web: «El hielo del planeta se está derritiendo»</t>
+          <t>Página web 1 (la primera que leíste)</t>
         </is>
       </c>
       <c r="B9" s="9" t="n"/>
@@ -791,7 +791,7 @@
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Página web: «Cambio climático: causas y evidencia observacional»</t>
+          <t>Página web 2 (la segunda que leíste)</t>
         </is>
       </c>
       <c r="B15" s="9" t="n"/>
@@ -818,7 +818,7 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Página web: «Forzamiento radiativo y sensibilidad climática»</t>
+          <t>Página web 3 (la tercera que leíste)</t>
         </is>
       </c>
       <c r="B21" s="9" t="n"/>
@@ -1861,7 +1861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1893,7 +1893,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Versión 3.0 — 29/09/2026</t>
+          <t>Basado en el Anexo 4 del protocolo (v3.0, 29/09/2026), adaptado a la lectura</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="42" t="inlineStr">
         <is>
-          <t>Considerando los 2 métodos, ¿cuál te pareció el más rápido? Por favor, ordénalos.</t>
+          <t>Considerando los 2 métodos, ¿con cuál la ayuda llegó en mejor momento? Por favor, ordénalos.</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="42" t="inlineStr">
         <is>
-          <t>¿Con cuál crees que cometiste menos errores (en orden)?</t>
+          <t>¿Con cuál método entendiste mejor el contenido (en orden)?</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="42" t="inlineStr">
         <is>
-          <t>Si tuvieras que usar un solo método para comunicarte, ¿cuál elegirías? Por favor, ordena:</t>
+          <t>Si tuvieras que leer textos difíciles con un solo método, ¿cuál elegirías? Por favor, ordena:</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="B44" s="40" t="inlineStr">
         <is>
-          <t>¿En qué medida la técnica te permitió mejorar tu rendimiento?</t>
+          <t>¿En qué medida el método te ayudó a entender el texto?</t>
         </is>
       </c>
       <c r="C44" s="27" t="n"/>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B45" s="41" t="inlineStr">
         <is>
-          <t>¿Hasta qué punto la técnica ha permitido una reducción en el número de errores cometidos?</t>
+          <t>¿Qué tan útiles fueron las explicaciones que recibiste?</t>
         </is>
       </c>
       <c r="C45" s="27" t="n"/>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B46" s="40" t="inlineStr">
         <is>
-          <t>¿En qué nivel resultaban más agradables de usar las interfaces con la técnica?</t>
+          <t>¿Qué tan agradable fue leer con este método?</t>
         </is>
       </c>
       <c r="C46" s="27" t="n"/>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B47" s="41" t="inlineStr">
         <is>
-          <t>¿Qué tan fácil fue aprender a utilizar esta técnica?</t>
+          <t>¿Qué tan fácil fue aprender a utilizar este método?</t>
         </is>
       </c>
       <c r="C47" s="27" t="n"/>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B48" s="40" t="inlineStr">
         <is>
-          <t>¿Qué tan precisa percibiste la técnica durante la interacción?</t>
+          <t>¿Con qué frecuencia la ayuda apareció cuando de verdad la necesitabas?</t>
         </is>
       </c>
       <c r="C48" s="27" t="n"/>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="B49" s="41" t="inlineStr">
         <is>
-          <t>¿Qué nivel de confianza sentiste al utilizar esta técnica?</t>
+          <t>¿Qué nivel de confianza sentiste al utilizar este método?</t>
         </is>
       </c>
       <c r="C49" s="27" t="n"/>
@@ -2235,91 +2235,103 @@
       </c>
       <c r="B50" s="40" t="inlineStr">
         <is>
-          <t>¿Qué tan dispuesto(a) estarías a utilizar esta técnica en tu vida diaria?</t>
+          <t>¿Qué tan dispuesto(a) estarías a utilizar este método en tu vida diaria al leer en internet?</t>
         </is>
       </c>
       <c r="C50" s="27" t="n"/>
       <c r="D50" s="27" t="n"/>
     </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="B51" s="41" t="inlineStr">
+        <is>
+          <t>¿Qué tanto te distrajo o interrumpió la ayuda?</t>
+        </is>
+      </c>
+      <c r="C51" s="27" t="n"/>
+      <c r="D51" s="27" t="n"/>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>Comentarios finales</t>
         </is>
       </c>
-      <c r="B52" s="9" t="n"/>
-      <c r="C52" s="9" t="n"/>
-      <c r="D52" s="9" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>¿Qué aspectos positivos encontraste en cada técnica?</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="70" customHeight="1">
-      <c r="A55" s="11" t="n"/>
-      <c r="B55" s="12" t="n"/>
-      <c r="C55" s="12" t="n"/>
-      <c r="D55" s="12" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="10" t="inlineStr">
+      <c r="B53" s="9" t="n"/>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="9" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>¿Qué aspectos positivos encontraste en cada método?</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="70" customHeight="1">
+      <c r="A56" s="11" t="n"/>
+      <c r="B56" s="12" t="n"/>
+      <c r="C56" s="12" t="n"/>
+      <c r="D56" s="12" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>¿Qué dificultades encontraste?</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="70" customHeight="1">
-      <c r="A58" s="11" t="n"/>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="10" t="inlineStr">
-        <is>
-          <t>¿Tienes alguna sugerencia para mejorar las técnicas evaluadas?</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="70" customHeight="1">
-      <c r="A61" s="11" t="n"/>
-      <c r="B61" s="12" t="n"/>
-      <c r="C61" s="12" t="n"/>
-      <c r="D61" s="12" t="n"/>
+    <row r="59" ht="70" customHeight="1">
+      <c r="A59" s="11" t="n"/>
+      <c r="B59" s="12" t="n"/>
+      <c r="C59" s="12" t="n"/>
+      <c r="D59" s="12" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>¿Tienes alguna sugerencia para mejorar los métodos evaluados?</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="70" customHeight="1">
+      <c r="A62" s="11" t="n"/>
+      <c r="B62" s="12" t="n"/>
+      <c r="C62" s="12" t="n"/>
+      <c r="D62" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A53:D53"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A62:D62"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A59:D59"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A60:D60"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A61:D61"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A54:D54"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A56:D56"/>
     <mergeCell ref="A21:D21"/>
     <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A57:D57"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C18 C19 C22 C23 C26 C27 C30 C31" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Elige una opción de la lista." promptTitle="Elige una opción" prompt="Usa la flecha ▼ de la derecha." type="list">
       <formula1>"1 = Primer lugar,2 = Segundo lugar"</formula1>
     </dataValidation>
-    <dataValidation sqref="C44 C45 C46 C47 C48 C49 C50 D44 D45 D46 D47 D48 D49 D50" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Elige una opción de la lista." promptTitle="Elige una opción" prompt="Usa la flecha ▼ de la derecha." type="list">
+    <dataValidation sqref="C44 C45 C46 C47 C48 C49 C50 C51 D44 D45 D46 D47 D48 D49 D50 D51" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Elige una opción de la lista." promptTitle="Elige una opción" prompt="Usa la flecha ▼ de la derecha." type="list">
       <formula1>"1 = Muy bajo,2 = Bajo,3 = Medio,4 = Alto,5 = Muy alto"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2335,7 +2347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2941,7 +2953,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>orden_rapido_m1</t>
+          <t>orden_momento_m1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2958,7 +2970,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>orden_rapido_m2</t>
+          <t>orden_momento_m2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3009,7 +3021,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>orden_errores_m1</t>
+          <t>orden_comprension_m1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3026,7 +3038,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>orden_errores_m2</t>
+          <t>orden_comprension_m2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3077,7 +3089,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>califica_rendimiento_m1</t>
+          <t>califica_entender_m1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3094,7 +3106,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>califica_rendimiento_m2</t>
+          <t>califica_entender_m2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3111,7 +3123,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>califica_menos_errores_m1</t>
+          <t>califica_utilidad_m1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3128,7 +3140,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>califica_menos_errores_m2</t>
+          <t>califica_utilidad_m2</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3213,7 +3225,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>califica_precision_m1</t>
+          <t>califica_oportuna_m1</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3230,7 +3242,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>califica_precision_m2</t>
+          <t>califica_oportuna_m2</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3315,12 +3327,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>comentario_positivos</t>
+          <t>califica_distraccion_m1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>A55</t>
+          <t>C51</t>
         </is>
       </c>
     </row>
@@ -3332,12 +3344,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>comentario_dificultades</t>
+          <t>califica_distraccion_m2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>A58</t>
+          <t>D51</t>
         </is>
       </c>
     </row>
@@ -3349,12 +3361,46 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
+          <t>comentario_positivos</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>A56</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Post-experimento</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>comentario_dificultades</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>A59</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Post-experimento</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>comentario_sugerencias</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>A61</t>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>A62</t>
         </is>
       </c>
     </row>

</xml_diff>